<commit_message>
Se modificó para que elimine los directorios duplicados en el xml
</commit_message>
<xml_diff>
--- a/Directorio_AMPYME.xlsx
+++ b/Directorio_AMPYME.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="261">
   <si>
     <t>Correspondencia</t>
   </si>
@@ -48,18 +48,6 @@
   </si>
   <si>
     <t>Contraloria</t>
-  </si>
-  <si>
-    <t>750-0741</t>
-  </si>
-  <si>
-    <t>750-0743</t>
-  </si>
-  <si>
-    <t>750-0740</t>
-  </si>
-  <si>
-    <t>520-1430</t>
   </si>
   <si>
     <t>Mantenimiento</t>
@@ -1285,21 +1273,21 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="B1" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="C1" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="10" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C2" s="1">
         <v>5249077</v>
@@ -1307,10 +1295,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="C3" s="1">
         <v>5005718</v>
@@ -1318,10 +1306,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="10" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C4" s="2">
         <v>5005774</v>
@@ -1329,10 +1317,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="C5" s="1">
         <v>5005750</v>
@@ -1340,10 +1328,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="11" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="C6" s="2">
         <v>5043940</v>
@@ -1351,10 +1339,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C7" s="2">
         <v>5005704</v>
@@ -1362,10 +1350,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C8" s="1">
         <v>3460277</v>
@@ -1373,10 +1361,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="11" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C9" s="1">
         <v>5005717</v>
@@ -1384,10 +1372,10 @@
     </row>
     <row r="10" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A10" s="10" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C10" s="9">
         <v>5005735</v>
@@ -1395,10 +1383,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C11" s="1">
         <v>5005720</v>
@@ -1406,10 +1394,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="10" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C12" s="1">
         <v>9261028</v>
@@ -1417,10 +1405,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="10" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C13" s="1">
         <v>5005705</v>
@@ -1428,10 +1416,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="10" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C14" s="2">
         <v>5043913</v>
@@ -1439,10 +1427,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="10" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C15" s="1">
         <v>5005730</v>
@@ -1450,10 +1438,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="10" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C16" s="2">
         <v>5005739</v>
@@ -1461,10 +1449,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="10" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C17" s="2">
         <v>5005732</v>
@@ -1472,10 +1460,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="10" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C18" s="1">
         <v>5005781</v>
@@ -1483,10 +1471,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="10" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C19" s="1">
         <v>5005755</v>
@@ -1494,10 +1482,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" s="11" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C20" s="1">
         <v>5043951</v>
@@ -1514,10 +1502,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" s="11" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C22" s="1">
         <v>5043910</v>
@@ -1525,7 +1513,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" s="10" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B23" s="1"/>
       <c r="C23" s="1">
@@ -1534,10 +1522,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" s="10" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C24" s="2">
         <v>5043946</v>
@@ -1545,10 +1533,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" s="10" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="C25" s="2">
         <v>5043937</v>
@@ -1556,10 +1544,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" s="10" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C26" s="1">
         <v>5249080</v>
@@ -1567,10 +1555,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" s="10" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C27" s="2">
         <v>5005734</v>
@@ -1578,10 +1566,10 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" s="10" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C28" s="2">
         <v>5005762</v>
@@ -1589,10 +1577,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" s="10" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C29" s="4">
         <v>5005700</v>
@@ -1600,16 +1588,16 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" s="10" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C30" s="2">
         <v>5043928</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="28" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" s="12" t="s">
         <v>0</v>
       </c>
@@ -1620,10 +1608,10 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" s="10" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C32" s="2">
         <v>5043963</v>
@@ -1631,21 +1619,21 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" s="10" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C33" s="1">
         <v>5005777</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="28" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" s="10" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C34" s="1">
         <v>5005770</v>
@@ -1653,10 +1641,10 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" s="10" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C35" s="1">
         <v>5005723</v>
@@ -1664,10 +1652,10 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" s="10" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C36" s="1">
         <v>4755176</v>
@@ -1675,10 +1663,10 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" s="10" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C37" s="1">
         <v>9351755</v>
@@ -1686,10 +1674,10 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" s="10" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C38" s="1">
         <v>3460273</v>
@@ -1697,10 +1685,10 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" s="10" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C39" s="2">
         <v>5043912</v>
@@ -1708,10 +1696,10 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" s="10" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C40" s="1">
         <v>9130755</v>
@@ -1719,32 +1707,32 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" s="10" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="C41" s="4">
         <v>7775861</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="28" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" s="10" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C42" s="2">
         <v>5005733</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="28" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" s="10" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="C43" s="2">
         <v>5043959</v>
@@ -1752,10 +1740,10 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" s="10" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C44" s="1">
         <v>5249971</v>
@@ -1763,10 +1751,10 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C45" s="1">
         <v>9351758</v>
@@ -1774,10 +1762,10 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" s="10" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C46" s="1">
         <v>5043926</v>
@@ -1785,10 +1773,10 @@
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" s="10" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C47" s="2">
         <v>5043917</v>
@@ -1796,10 +1784,10 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" s="10" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C48" s="2">
         <v>5005751</v>
@@ -1807,10 +1795,10 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" s="10" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="C49" s="1">
         <v>5045756</v>
@@ -1818,10 +1806,10 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" s="10" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C50" s="2">
         <v>5005794</v>
@@ -1829,10 +1817,10 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" s="10" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C51" s="2">
         <v>5005722</v>
@@ -1840,10 +1828,10 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" s="11" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C52" s="5">
         <v>5005726</v>
@@ -1851,10 +1839,10 @@
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" s="10" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C53" s="1">
         <v>9261026</v>
@@ -1862,10 +1850,10 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" s="10" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C54" s="1">
         <v>3460274</v>
@@ -1873,10 +1861,10 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" s="10" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="C55" s="2">
         <v>5005714</v>
@@ -1884,10 +1872,10 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A56" s="10" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C56" s="4">
         <v>7775862</v>
@@ -1895,10 +1883,10 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A57" s="10" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C57" s="1">
         <v>5005759</v>
@@ -1906,10 +1894,10 @@
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" s="10" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C58" s="2">
         <v>5043934</v>
@@ -1917,32 +1905,32 @@
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A59" s="10" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C59" s="4">
         <v>7775646</v>
       </c>
     </row>
-    <row r="60" spans="1:3" ht="28" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" s="10" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="B60" s="13" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="C60" s="2">
         <v>5043920</v>
       </c>
     </row>
-    <row r="61" spans="1:3" ht="42" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A61" s="14" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="B61" s="13" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="C61" s="2">
         <v>5005708</v>
@@ -1950,21 +1938,21 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A62" s="15" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>237</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>10</v>
+        <v>233</v>
+      </c>
+      <c r="C62" s="6">
+        <v>7500740</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A63" s="11" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="C63" s="1">
         <v>5043908</v>
@@ -1972,10 +1960,10 @@
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A64" s="10" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C64" s="1">
         <v>5043919</v>
@@ -1983,10 +1971,10 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A65" s="10" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C65" s="1">
         <v>5043962</v>
@@ -1994,10 +1982,10 @@
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A66" s="16" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C66" s="2">
         <v>5005721</v>
@@ -2005,10 +1993,10 @@
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A67" s="10" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C67" s="2">
         <v>5043927</v>
@@ -2016,10 +2004,10 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A68" s="10" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C68" s="2">
         <v>5005712</v>
@@ -2027,10 +2015,10 @@
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A69" s="10" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C69" s="4">
         <v>7500744</v>
@@ -2038,10 +2026,10 @@
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A70" s="10" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C70" s="1">
         <v>3460283</v>
@@ -2049,10 +2037,10 @@
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A71" s="10" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C71" s="2">
         <v>5005711</v>
@@ -2060,10 +2048,10 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A72" s="10" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C72" s="2">
         <v>5005703</v>
@@ -2071,10 +2059,10 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A73" s="10" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C73" s="1">
         <v>9061522</v>
@@ -2082,10 +2070,10 @@
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A74" s="10" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C74" s="2">
         <v>5005748</v>
@@ -2093,10 +2081,10 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A75" s="10" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C75" s="1" t="s">
         <v>6</v>
@@ -2104,10 +2092,10 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A76" s="10" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="C76" s="2">
         <v>5005753</v>
@@ -2115,10 +2103,10 @@
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A77" s="10" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="C77" s="1">
         <v>9261029</v>
@@ -2126,10 +2114,10 @@
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A78" s="10" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C78" s="1">
         <v>5005798</v>
@@ -2137,10 +2125,10 @@
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A79" s="10" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C79" s="2">
         <v>5005775</v>
@@ -2148,10 +2136,10 @@
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A80" s="17" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C80" s="1">
         <v>5005779</v>
@@ -2159,10 +2147,10 @@
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A81" s="11" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C81" s="3">
         <v>5005795</v>
@@ -2170,10 +2158,10 @@
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A82" s="10" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C82" s="2">
         <v>5043909</v>
@@ -2181,10 +2169,10 @@
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A83" s="11" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C83" s="1">
         <v>5043911</v>
@@ -2192,10 +2180,10 @@
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A84" s="10" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C84" s="1">
         <v>3460280</v>
@@ -2203,10 +2191,10 @@
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A85" s="10" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="C85" s="2">
         <v>5005758</v>
@@ -2223,21 +2211,21 @@
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A87" s="15" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B87" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="C87" s="6" t="s">
-        <v>9</v>
+        <v>138</v>
+      </c>
+      <c r="C87" s="6">
+        <v>7500743</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A88" s="10" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C88" s="1">
         <v>5243539</v>
@@ -2245,10 +2233,10 @@
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A89" s="10" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C89" s="4">
         <v>7775643</v>
@@ -2256,10 +2244,10 @@
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A90" s="10" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="C90" s="2">
         <v>5005780</v>
@@ -2267,10 +2255,10 @@
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A91" s="10" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="C91" s="1">
         <v>9351759</v>
@@ -2278,10 +2266,10 @@
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A92" s="10" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C92" s="2">
         <v>5005724</v>
@@ -2289,10 +2277,10 @@
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A93" s="10" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C93" s="1">
         <v>5201427</v>
@@ -2300,21 +2288,21 @@
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A94" s="10" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="C94" s="1" t="s">
-        <v>8</v>
+        <v>149</v>
+      </c>
+      <c r="C94" s="1">
+        <v>7500741</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A95" s="10" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="C95" s="2">
         <v>5005760</v>
@@ -2322,10 +2310,10 @@
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A96" s="10" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="C96" s="2">
         <v>5005761</v>
@@ -2333,10 +2321,10 @@
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A97" s="10" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="C97" s="1">
         <v>3460282</v>
@@ -2344,10 +2332,10 @@
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A98" s="10" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C98" s="1">
         <v>9351757</v>
@@ -2364,10 +2352,10 @@
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A100" s="10" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C100" s="4">
         <v>7500745</v>
@@ -2375,10 +2363,10 @@
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A101" s="10" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C101" s="1">
         <v>3460279</v>
@@ -2386,7 +2374,7 @@
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A102" s="10" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B102" s="2"/>
       <c r="C102" s="2">
@@ -2395,10 +2383,10 @@
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A103" s="10" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C103" s="1">
         <v>5201429</v>
@@ -2406,10 +2394,10 @@
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A104" s="17" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C104" s="1">
         <v>5043938</v>
@@ -2417,10 +2405,10 @@
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A105" s="10" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C105" s="1">
         <v>9130756</v>
@@ -2428,10 +2416,10 @@
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A106" s="12" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C106" s="1">
         <v>5005773</v>
@@ -2439,10 +2427,10 @@
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A107" s="10" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C107" s="2">
         <v>5005776</v>
@@ -2450,10 +2438,10 @@
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A108" s="10" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C108" s="2">
         <v>5005782</v>
@@ -2461,21 +2449,21 @@
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A109" s="10" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="C109" s="1" t="s">
-        <v>11</v>
+        <v>121</v>
+      </c>
+      <c r="C109" s="1">
+        <v>5201430</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A110" s="11" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="C110" s="1">
         <v>5005799</v>
@@ -2483,10 +2471,10 @@
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A111" s="10" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C111" s="2">
         <v>5005746</v>
@@ -2494,10 +2482,10 @@
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A112" s="10" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C112" s="1">
         <v>9060608</v>
@@ -2505,10 +2493,10 @@
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A113" s="10" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C113" s="2">
         <v>5005715</v>
@@ -2516,7 +2504,7 @@
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A114" s="10" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B114" s="1"/>
       <c r="C114" s="1">
@@ -2525,10 +2513,10 @@
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A115" s="10" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="C115" s="2">
         <v>5005716</v>
@@ -2536,10 +2524,10 @@
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A116" s="11" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C116" s="1">
         <v>5005747</v>
@@ -2547,10 +2535,10 @@
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A117" s="10" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C117" s="2">
         <v>5043960</v>
@@ -2558,10 +2546,10 @@
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A118" s="10" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="C118" s="1">
         <v>7775644</v>
@@ -2569,10 +2557,10 @@
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A119" s="10" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="C119" s="2">
         <v>5005745</v>
@@ -2580,10 +2568,10 @@
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A120" s="10" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="C120" s="1">
         <v>3460278</v>
@@ -2591,10 +2579,10 @@
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A121" s="10" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C121" s="1">
         <v>9261025</v>
@@ -2602,10 +2590,10 @@
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A122" s="10" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="C122" s="1">
         <v>5249037</v>
@@ -2613,10 +2601,10 @@
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A123" s="10" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C123" s="2">
         <v>5005729</v>
@@ -2624,10 +2612,10 @@
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A124" s="10" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="C124" s="2">
         <v>5005771</v>
@@ -2635,10 +2623,10 @@
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A125" s="10" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="C125" s="2">
         <v>5005788</v>
@@ -2646,16 +2634,16 @@
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A126" s="10" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="C126" s="2">
         <v>5043958</v>
       </c>
     </row>
-    <row r="127" spans="1:3" ht="28" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A127" s="10" t="s">
         <v>3</v>
       </c>
@@ -2666,10 +2654,10 @@
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A128" s="10" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="C128" s="2">
         <v>5043921</v>
@@ -2677,10 +2665,10 @@
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A129" s="12" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="C129" s="1">
         <v>5043922</v>
@@ -2688,10 +2676,10 @@
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A130" s="10" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="C130" s="2">
         <v>5005742</v>
@@ -2699,10 +2687,10 @@
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A131" s="10" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C131" s="2">
         <v>5005731</v>
@@ -2710,10 +2698,10 @@
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A132" s="10" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="C132" s="1">
         <v>5005707</v>
@@ -2721,10 +2709,10 @@
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A133" s="10" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="C133" s="4">
         <v>7500741</v>
@@ -2732,10 +2720,10 @@
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A134" s="10" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="C134" s="4">
         <v>7500743</v>
@@ -2743,10 +2731,10 @@
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A135" s="10" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="C135" s="1">
         <v>9060609</v>
@@ -2754,10 +2742,10 @@
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A136" s="10" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C136" s="4">
         <v>7775641</v>
@@ -2765,10 +2753,10 @@
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A137" s="10" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C137" s="4">
         <v>7775642</v>
@@ -2776,10 +2764,10 @@
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A138" s="10" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C138" s="4">
         <v>7775644</v>
@@ -2787,10 +2775,10 @@
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A139" s="10" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C139" s="4">
         <v>7775645</v>
@@ -2798,10 +2786,10 @@
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A140" s="18" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B140" s="7" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="C140" s="7">
         <v>2870307</v>
@@ -2809,10 +2797,10 @@
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A141" s="10" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B141" s="4" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C141" s="4">
         <v>7775864</v>
@@ -2820,10 +2808,10 @@
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A142" s="10" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="C142" s="1">
         <v>4755177</v>
@@ -2831,10 +2819,10 @@
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A143" s="10" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B143" s="4" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C143" s="4">
         <v>7775863</v>
@@ -2842,10 +2830,10 @@
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A144" s="10" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="C144" s="1">
         <v>9351754</v>
@@ -2853,10 +2841,10 @@
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A145" s="10" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="C145" s="1">
         <v>5201428</v>
@@ -2864,27 +2852,27 @@
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A146" s="10" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C146" s="2">
         <v>5043918</v>
       </c>
     </row>
-    <row r="147" spans="1:3" ht="42" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A147" s="10" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="B147" s="2"/>
       <c r="C147" s="2">
         <v>5005737</v>
       </c>
     </row>
-    <row r="148" spans="1:3" ht="42" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A148" s="10" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="B148" s="1"/>
       <c r="C148" s="1">
@@ -2902,10 +2890,10 @@
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A150" s="10" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="C150" s="2">
         <v>5005749</v>
@@ -2913,10 +2901,10 @@
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A151" s="10" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="C151" s="1">
         <v>9130760</v>
@@ -2924,10 +2912,10 @@
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A152" s="10" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="C152" s="2">
         <v>5005757</v>
@@ -2944,10 +2932,10 @@
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A154" s="10" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="C154" s="1">
         <v>9130758</v>
@@ -2964,10 +2952,10 @@
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A156" s="11" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B156" s="1" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="C156" s="1">
         <v>5005768</v>
@@ -2975,18 +2963,18 @@
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A157" s="10" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C157" s="2">
         <v>5005725</v>
       </c>
     </row>
-    <row r="158" spans="1:3" ht="28" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A158" s="10" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B158" s="1"/>
       <c r="C158" s="1">
@@ -2995,10 +2983,10 @@
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A159" s="10" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="C159" s="2">
         <v>5043948</v>
@@ -3006,10 +2994,10 @@
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A160" s="10" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="C160" s="1">
         <v>4754767</v>
@@ -3017,7 +3005,7 @@
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A161" s="10" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B161" s="1"/>
       <c r="C161" s="1">
@@ -3026,10 +3014,10 @@
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A162" s="10" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C162" s="2">
         <v>5043960</v>
@@ -3037,10 +3025,10 @@
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A163" s="10" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C163" s="2">
         <v>5005783</v>
@@ -3048,10 +3036,10 @@
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A164" s="11" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="C164" s="1">
         <v>5043929</v>
@@ -3059,10 +3047,10 @@
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A165" s="10" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="C165" s="2">
         <v>5005778</v>
@@ -3070,10 +3058,10 @@
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A166" s="10" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C166" s="2">
         <v>5043964</v>
@@ -3081,10 +3069,10 @@
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A167" s="10" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="B167" s="1" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="C167" s="1">
         <v>9261027</v>
@@ -3092,10 +3080,10 @@
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A168" s="10" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="B168" s="1" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="C168" s="1">
         <v>9130757</v>
@@ -3103,10 +3091,10 @@
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A169" s="10" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C169" s="2">
         <v>5005789</v>
@@ -3114,18 +3102,18 @@
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A170" s="11" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="B170" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C170" s="1">
         <v>5043952</v>
       </c>
     </row>
-    <row r="171" spans="1:3" ht="56" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A171" s="19" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="B171" s="8"/>
       <c r="C171" s="8">

</xml_diff>